<commit_message>
se continuo realizando la division de metricas de pc, android y esp32
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cartu\OneDrive\Escritorio\Nueva carpeta (2)\automatizacion_completa\datos_entrada\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\medidor de metricas\automatizacion_completa\datos_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828C7543-17B3-43B7-8862-C59F1DC86B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E109A8A8-1976-4381-8FF2-AD2EA3DEC5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -245,7 +245,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -304,6 +304,8 @@
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -517,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="16.453125" customWidth="1"/>
@@ -837,6 +839,22 @@
       <c r="K11" s="21">
         <v>16384</v>
       </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="F12" s="22"/>
+      <c r="H12" s="22"/>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="F13" s="22"/>
+      <c r="H13" s="22"/>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="F14" s="23"/>
+      <c r="H14" s="22"/>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="F15" s="23"/>
+      <c r="H15" s="22"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>

<commit_message>
se agregaron proyectos del 2° cuatrimeteste del 2026 de Prog-Concurrente
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\medidor de metricas\automatizacion_completa\datos_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E109A8A8-1976-4381-8FF2-AD2EA3DEC5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4D433C-A82D-49C5-89D8-E02024F4C895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="CPU_Memoria" sheetId="1" r:id="rId1"/>
     <sheet name="Concurrencia" sheetId="4" r:id="rId2"/>
     <sheet name="Datos Tokens" sheetId="5" r:id="rId3"/>
+    <sheet name="Funcionalidad" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="57">
   <si>
     <t>Codigo</t>
   </si>
@@ -44,36 +45,6 @@
     <t>Refinamientos</t>
   </si>
   <si>
-    <t>M1</t>
-  </si>
-  <si>
-    <t>M2</t>
-  </si>
-  <si>
-    <t>M3-CC-Haiku</t>
-  </si>
-  <si>
-    <t>M3-CC-Opus</t>
-  </si>
-  <si>
-    <t>M4-IDE-Gemini</t>
-  </si>
-  <si>
-    <t>M4-IDE-Sonnet</t>
-  </si>
-  <si>
-    <t>M4-IDE-GPT</t>
-  </si>
-  <si>
-    <t>M4-IDE-Deepseek</t>
-  </si>
-  <si>
-    <t>M5</t>
-  </si>
-  <si>
-    <t>M6</t>
-  </si>
-  <si>
     <t>Sincronizacion correcta</t>
   </si>
   <si>
@@ -150,6 +121,93 @@
   </si>
   <si>
     <t>Memoria Acc2 (MB)</t>
+  </si>
+  <si>
+    <t>1C-26-M1</t>
+  </si>
+  <si>
+    <t>1C-26-M3-CC-Haiku</t>
+  </si>
+  <si>
+    <t>1C-26-M2</t>
+  </si>
+  <si>
+    <t>1C-26-M3-CC-Opus</t>
+  </si>
+  <si>
+    <t>1C-26-M4-IDE-Gemini</t>
+  </si>
+  <si>
+    <t>1C-26-M4-IDE-Sonnet</t>
+  </si>
+  <si>
+    <t>1C-26-M4-IDE-GPT</t>
+  </si>
+  <si>
+    <t>1C-26-M4-IDE-Deepseek</t>
+  </si>
+  <si>
+    <t>1C-26-M5</t>
+  </si>
+  <si>
+    <t>1C-26-M6</t>
+  </si>
+  <si>
+    <t>2C-26-M6</t>
+  </si>
+  <si>
+    <t>2C-26-M1</t>
+  </si>
+  <si>
+    <t>2C-26-M2</t>
+  </si>
+  <si>
+    <t>2C-26-M3</t>
+  </si>
+  <si>
+    <t>2C-26-M4</t>
+  </si>
+  <si>
+    <t>2C-26-M5</t>
+  </si>
+  <si>
+    <t>2C-26-M7</t>
+  </si>
+  <si>
+    <t>2C-26-M8</t>
+  </si>
+  <si>
+    <t>2C-26-M9</t>
+  </si>
+  <si>
+    <t>simulación con baja carga: 50 aviones, 30 vuelos, 10 hilos para asignación (60seg de duración)</t>
+  </si>
+  <si>
+    <t>simulación con mayor carga: 500 aviones, 1000 vuelos, 200 hilos para asignación (60seg de duración)</t>
+  </si>
+  <si>
+    <t>Funciona sin errores</t>
+  </si>
+  <si>
+    <t>Cumple objetivo funcional</t>
+  </si>
+  <si>
+    <t>Diseño de la app</t>
+  </si>
+  <si>
+    <t>HTTP secuencial, 1 solicitud simultánea durante 30 s</t>
+  </si>
+  <si>
+    <t>HTTP concurrente, 32 solicitudes simultáneas durante 30 s</t>
+  </si>
+  <si>
+    <t>ps util +jmh</t>
+  </si>
+  <si>
+    <t>Ejecución secuencial</t>
+  </si>
+  <si>
+    <t>Ejecución concurrente</t>
   </si>
 </sst>
 </file>
@@ -159,7 +217,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,6 +240,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -193,11 +257,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
       </patternFill>
     </fill>
     <fill>
@@ -222,6 +281,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -241,11 +306,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -259,7 +325,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -270,46 +335,86 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{0352F441-D3BB-49AE-B4AD-2AF916746F23}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -519,16 +624,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="1" max="1" width="22.36328125" customWidth="1"/>
     <col min="2" max="2" width="12.54296875" customWidth="1"/>
     <col min="3" max="3" width="23.08984375" customWidth="1"/>
     <col min="4" max="4" width="13.453125" customWidth="1"/>
-    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="5" max="5" width="30.453125" customWidth="1"/>
     <col min="6" max="6" width="14.7265625" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="7" max="7" width="39.81640625" customWidth="1"/>
     <col min="8" max="8" width="22.90625" customWidth="1"/>
     <col min="9" max="9" width="13.453125" customWidth="1"/>
     <col min="10" max="10" width="12.36328125" customWidth="1"/>
@@ -536,333 +641,518 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="28">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="G1" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="J1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>33</v>
+      <c r="K1" s="9" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="11">
+        <v>28</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="10">
         <v>4</v>
       </c>
-      <c r="E2" s="11"/>
-      <c r="F2" s="12">
+      <c r="E2" s="10"/>
+      <c r="F2" s="11">
         <v>0.04</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="17">
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="16">
         <v>52</v>
       </c>
-      <c r="J2" s="18"/>
-      <c r="K2" s="21">
+      <c r="J2" s="17"/>
+      <c r="K2" s="20">
         <v>4096</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="11">
+      <c r="B3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="10">
         <v>8</v>
       </c>
-      <c r="E3" s="11"/>
-      <c r="F3" s="12">
+      <c r="E3" s="10"/>
+      <c r="F3" s="11">
         <v>0.5</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="17">
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="16">
         <v>68</v>
       </c>
-      <c r="J3" s="18"/>
-      <c r="K3" s="21">
+      <c r="J3" s="17"/>
+      <c r="K3" s="20">
         <v>4096</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="11">
+      <c r="B4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="10">
         <v>8</v>
       </c>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12">
+      <c r="E4" s="10"/>
+      <c r="F4" s="11">
         <v>0.42</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="17">
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="16">
         <v>238</v>
       </c>
-      <c r="J4" s="18"/>
-      <c r="K4" s="21">
+      <c r="J4" s="17"/>
+      <c r="K4" s="20">
         <v>8192</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="11">
+        <v>31</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="10">
         <v>8</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="12">
+      <c r="E5" s="10"/>
+      <c r="F5" s="11">
         <v>0.42</v>
       </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="17">
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="16">
         <v>238</v>
       </c>
-      <c r="J5" s="18"/>
-      <c r="K5" s="21">
+      <c r="J5" s="17"/>
+      <c r="K5" s="20">
         <v>8192</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="11">
+        <v>32</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="10">
         <v>4</v>
       </c>
-      <c r="E6" s="11"/>
-      <c r="F6" s="14">
+      <c r="E6" s="10"/>
+      <c r="F6" s="13">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="19">
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="18">
         <v>20</v>
       </c>
-      <c r="J6" s="18"/>
-      <c r="K6" s="21">
+      <c r="J6" s="17"/>
+      <c r="K6" s="20">
         <v>4096</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="11">
+        <v>33</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="10">
         <v>4</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="14">
+      <c r="E7" s="10"/>
+      <c r="F7" s="13">
         <v>2E-3</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="17">
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="16">
         <v>15</v>
       </c>
-      <c r="J7" s="18"/>
-      <c r="K7" s="21">
+      <c r="J7" s="17"/>
+      <c r="K7" s="20">
         <v>4096</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="11">
+        <v>34</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="10">
         <v>4</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="15">
+      <c r="E8" s="10"/>
+      <c r="F8" s="14">
         <v>0.1061</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="17">
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="16">
         <v>20</v>
       </c>
-      <c r="J8" s="18"/>
-      <c r="K8" s="21">
+      <c r="J8" s="17"/>
+      <c r="K8" s="20">
         <v>4096</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="11">
+        <v>35</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="10">
         <v>8</v>
       </c>
-      <c r="E9" s="11"/>
-      <c r="F9" s="15">
+      <c r="E9" s="10"/>
+      <c r="F9" s="14">
         <v>0.12429999999999999</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="17">
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="16">
         <v>20</v>
       </c>
-      <c r="J9" s="18"/>
-      <c r="K9" s="21">
+      <c r="J9" s="17"/>
+      <c r="K9" s="20">
         <v>4096</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="11">
+        <v>36</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="10">
         <v>8</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="14">
+      <c r="E10" s="10"/>
+      <c r="F10" s="13">
         <v>2.0333000000000001</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="20">
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="19">
         <v>200</v>
       </c>
-      <c r="J10" s="18"/>
-      <c r="K10" s="21">
+      <c r="J10" s="17"/>
+      <c r="K10" s="20">
         <v>8192</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="11">
+        <v>37</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="10">
         <v>8</v>
       </c>
-      <c r="E11" s="11"/>
-      <c r="F11" s="16">
+      <c r="E11" s="10"/>
+      <c r="F11" s="15">
         <v>3.04</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="17">
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="16">
         <v>396</v>
       </c>
-      <c r="J11" s="18"/>
-      <c r="K11" s="21">
+      <c r="J11" s="17"/>
+      <c r="K11" s="20">
         <v>16384</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="F12" s="22"/>
-      <c r="H12" s="22"/>
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="20"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="F13" s="22"/>
-      <c r="H13" s="22"/>
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="10">
+        <v>12</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="F13" s="14">
+        <v>0.55300000000000005</v>
+      </c>
+      <c r="G13" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="H13" s="12">
+        <v>0.73670000000000002</v>
+      </c>
+      <c r="I13" s="19">
+        <v>177.82</v>
+      </c>
+      <c r="J13" s="17">
+        <v>177.83</v>
+      </c>
+      <c r="K13" s="20">
+        <v>16108</v>
+      </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="F14" s="23"/>
-      <c r="H14" s="22"/>
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="20"/>
     </row>
     <row r="15" spans="1:11">
-      <c r="F15" s="23"/>
-      <c r="H15" s="22"/>
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="19"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="20"/>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="20"/>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="10">
+        <v>10</v>
+      </c>
+      <c r="E17" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0.1303</v>
+      </c>
+      <c r="G17" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="H17" s="12">
+        <v>1.0186999999999999</v>
+      </c>
+      <c r="I17" s="19">
+        <v>25.91</v>
+      </c>
+      <c r="J17" s="17">
+        <v>49.28</v>
+      </c>
+      <c r="K17" s="20">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="10">
+        <v>8</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0.15409999999999999</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="H18" s="12">
+        <v>0.19289999999999999</v>
+      </c>
+      <c r="I18" s="19">
+        <v>25.71</v>
+      </c>
+      <c r="J18" s="17">
+        <v>25.9</v>
+      </c>
+      <c r="K18" s="20">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="20"/>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="B21" s="10"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" sqref="C2:C11" xr:uid="{C300DFF5-46E8-4F25-B753-4EE6C8F7C280}">
+  <dataValidations count="3">
+    <dataValidation type="list" sqref="C2:C12 C14:C20" xr:uid="{C300DFF5-46E8-4F25-B753-4EE6C8F7C280}">
       <formula1>"100%=1 núcleo,100%=capacidad total"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B2:B11" xr:uid="{1AD00D99-B2BA-4FAF-B153-E405C90E461E}">
+    <dataValidation type="list" sqref="B2:B21" xr:uid="{1AD00D99-B2BA-4FAF-B153-E405C90E461E}">
       <formula1>"psutil,ps + jcmd,ps,Otro"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C13" xr:uid="{4B57103C-9F02-483C-9123-35C9E0AB2911}">
+      <formula1>"100%=1 núcleo,100%=capacidad total"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -872,10 +1162,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
+    <col min="1" max="1" width="21.1796875" customWidth="1"/>
     <col min="2" max="2" width="28.08984375" customWidth="1"/>
     <col min="3" max="3" width="26.90625" customWidth="1"/>
     <col min="4" max="4" width="38.26953125" customWidth="1"/>
@@ -887,190 +1177,268 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>16</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="5"/>
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1079,10 +1447,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="17.81640625" customWidth="1"/>
+    <col min="1" max="1" width="23.08984375" customWidth="1"/>
     <col min="2" max="2" width="20.6328125" customWidth="1"/>
     <col min="3" max="3" width="16.54296875" customWidth="1"/>
     <col min="4" max="4" width="17.1796875" customWidth="1"/>
@@ -1090,24 +1458,24 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
-        <v>23</v>
+      <c r="D1" s="8" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>18</v>
+        <v>28</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="C2" s="1">
         <v>3</v>
@@ -1118,12 +1486,12 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="7">
+        <v>9</v>
+      </c>
+      <c r="C3" s="6">
         <v>9</v>
       </c>
       <c r="D3" s="1">
@@ -1132,10 +1500,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
@@ -1146,10 +1514,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1">
         <v>2</v>
@@ -1160,10 +1528,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -1174,10 +1542,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1">
         <v>1</v>
@@ -1188,10 +1556,10 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
@@ -1202,10 +1570,10 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -1216,10 +1584,10 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" t="s">
         <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
       </c>
       <c r="C10">
         <v>80</v>
@@ -1230,16 +1598,270 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
         <v>2216</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="26">
+        <v>1</v>
+      </c>
+      <c r="D13" s="27">
+        <v>3500000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="24">
+        <v>3</v>
+      </c>
+      <c r="D17" s="24">
+        <v>160787</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18" s="35">
+        <v>86900</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49169CDD-39DA-43A4-BA10-B1D9578FCAE5}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="21.1796875" customWidth="1"/>
+    <col min="2" max="2" width="28.08984375" customWidth="1"/>
+    <col min="3" max="3" width="26.90625" customWidth="1"/>
+    <col min="4" max="4" width="38.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se agrego otro proyecto de programacion concurrente del 2° Cuatrimestre del 2026
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\medidor de metricas\automatizacion_completa\datos_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4D433C-A82D-49C5-89D8-E02024F4C895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5363EFB8-9A8C-4D7F-A5F6-CC104CF7243D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU_Memoria" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="61">
   <si>
     <t>Codigo</t>
   </si>
@@ -208,14 +208,27 @@
   </si>
   <si>
     <t>Ejecución concurrente</t>
+  </si>
+  <si>
+    <t>Otro</t>
+  </si>
+  <si>
+    <t>100%=capacidad total</t>
+  </si>
+  <si>
+    <t>Registro de 4 órdenes</t>
+  </si>
+  <si>
+    <t>Simulación concurrente de 100 órdenes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -247,7 +260,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -287,6 +300,18 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FF00B050"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -311,7 +336,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -409,6 +434,37 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1129,16 +1185,36 @@
       <c r="A20" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="20"/>
+      <c r="B20" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="36">
+        <v>16</v>
+      </c>
+      <c r="E20" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" s="37">
+        <v>3.2829999999999999E-3</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" s="39">
+        <v>6.8992999999999999E-2</v>
+      </c>
+      <c r="I20" s="40">
+        <v>272.11</v>
+      </c>
+      <c r="J20" s="41">
+        <v>487.14</v>
+      </c>
+      <c r="K20" s="42">
+        <v>34222.300000000003</v>
+      </c>
     </row>
     <row r="21" spans="1:11">
       <c r="B21" s="10"/>
@@ -1439,6 +1515,18 @@
       <c r="A20" t="s">
         <v>46</v>
       </c>
+      <c r="B20" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1681,6 +1769,15 @@
       <c r="A20" t="s">
         <v>46</v>
       </c>
+      <c r="B20" s="44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="45">
+        <v>10</v>
+      </c>
+      <c r="D20" s="45">
+        <v>47577</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1863,6 +1960,15 @@
       <c r="A20" t="s">
         <v>46</v>
       </c>
+      <c r="B20" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="46" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
se agregaron otros proyectos del 2° cuatrimestre de programacion concurrente
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\medidor de metricas\automatizacion_completa\datos_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5363EFB8-9A8C-4D7F-A5F6-CC104CF7243D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010CA5AE-4F4B-4F5E-B6A4-7839BC2EFF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="73">
   <si>
     <t>Codigo</t>
   </si>
@@ -162,9 +162,6 @@
     <t>2C-26-M2</t>
   </si>
   <si>
-    <t>2C-26-M3</t>
-  </si>
-  <si>
     <t>2C-26-M4</t>
   </si>
   <si>
@@ -220,15 +217,57 @@
   </si>
   <si>
     <t>Simulación concurrente de 100 órdenes</t>
+  </si>
+  <si>
+    <t>Simulación default: 2 camiones / 3 operarios (20 s × 3)</t>
+  </si>
+  <si>
+    <t>Estrés: 50 camiones / 50 operarios (20 s × 3)</t>
+  </si>
+  <si>
+    <t>Estimación por caracteres
+Reporte /cost
+Comando /context de</t>
+  </si>
+  <si>
+    <t>2C-26-M3-AN-Gemini</t>
+  </si>
+  <si>
+    <t>2C-26-M3-CC-Opus</t>
+  </si>
+  <si>
+    <t>2C-26-M3-CC-Composer</t>
+  </si>
+  <si>
+    <t>Carga Distribuida</t>
+  </si>
+  <si>
+    <t>Alta Conteción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.5% </t>
+  </si>
+  <si>
+    <t xml:space="preserve">62.6% </t>
+  </si>
+  <si>
+    <t>121.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">133.5% </t>
+  </si>
+  <si>
+    <t>114.2%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="0.0000%"/>
+    <numFmt numFmtId="164" formatCode="0.0000%"/>
+    <numFmt numFmtId="168" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -331,12 +370,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -438,13 +479,13 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="7" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -466,9 +507,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="5">
     <cellStyle name="Millares" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Millares 2" xfId="3" xr:uid="{C5AA9BD5-CEF8-4E4C-AD7A-A41F277842E7}"/>
+    <cellStyle name="Millares 3" xfId="4" xr:uid="{FF52AADE-9C35-4158-BE53-F76058096985}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{0352F441-D3BB-49AE-B4AD-2AF916746F23}"/>
   </cellStyles>
@@ -680,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="22.36328125" customWidth="1"/>
@@ -1021,7 +1087,7 @@
         <v>40</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" s="28" t="s">
         <v>20</v>
@@ -1030,13 +1096,13 @@
         <v>12</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F13" s="14">
         <v>0.55300000000000005</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H13" s="12">
         <v>0.73670000000000002</v>
@@ -1053,181 +1119,291 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="20"/>
+        <v>63</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="10">
+        <v>16</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="52" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" s="12">
+        <v>0.06</v>
+      </c>
+      <c r="I14" s="19">
+        <v>35</v>
+      </c>
+      <c r="J14" s="17">
+        <v>35</v>
+      </c>
+      <c r="K14" s="20">
+        <v>32660</v>
+      </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="20"/>
+        <v>64</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="10">
+        <v>16</v>
+      </c>
+      <c r="E15" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="G15" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="H15" s="54" t="s">
+        <v>72</v>
+      </c>
+      <c r="I15" s="19">
+        <v>72.77</v>
+      </c>
+      <c r="J15" s="17">
+        <v>77.22</v>
+      </c>
+      <c r="K15" s="20">
+        <v>32660</v>
+      </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="17"/>
-      <c r="K16" s="20"/>
+        <v>65</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="10">
+        <v>16</v>
+      </c>
+      <c r="E16" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="52" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="19">
+        <v>257.5</v>
+      </c>
+      <c r="J16" s="17">
+        <v>258.02999999999997</v>
+      </c>
+      <c r="K16" s="20">
+        <v>32660</v>
+      </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="10">
-        <v>10</v>
+      <c r="D17" s="32">
+        <v>16</v>
       </c>
       <c r="E17" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17" s="14">
-        <v>0.1303</v>
-      </c>
-      <c r="G17" s="33" t="s">
-        <v>48</v>
+        <v>60</v>
+      </c>
+      <c r="F17" s="52">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="G17" s="32" t="s">
+        <v>61</v>
       </c>
       <c r="H17" s="12">
-        <v>1.0186999999999999</v>
-      </c>
-      <c r="I17" s="19">
-        <v>25.91</v>
-      </c>
-      <c r="J17" s="17">
-        <v>49.28</v>
-      </c>
-      <c r="K17" s="20">
-        <v>16384</v>
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="I17" s="47">
+        <v>15.33</v>
+      </c>
+      <c r="J17" s="49">
+        <v>17.21</v>
+      </c>
+      <c r="K17" s="53">
+        <v>16176</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18" s="10">
-        <v>8</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F18" s="14">
-        <v>0.15409999999999999</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="H18" s="12">
-        <v>0.19289999999999999</v>
-      </c>
-      <c r="I18" s="19">
-        <v>25.71</v>
-      </c>
-      <c r="J18" s="17">
-        <v>25.9</v>
-      </c>
-      <c r="K18" s="20">
-        <v>16384</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="20"/>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="20"/>
+        <v>38</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="10">
+        <v>10</v>
+      </c>
+      <c r="E19" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0.1303</v>
+      </c>
+      <c r="G19" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="12">
+        <v>1.0186999999999999</v>
+      </c>
+      <c r="I19" s="19">
+        <v>25.91</v>
+      </c>
+      <c r="J19" s="17">
+        <v>49.28</v>
+      </c>
+      <c r="K19" s="20">
+        <v>16384</v>
+      </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="10">
+        <v>8</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="14">
+        <v>0.15409999999999999</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="H20" s="12">
+        <v>0.19289999999999999</v>
+      </c>
+      <c r="I20" s="19">
+        <v>25.71</v>
+      </c>
+      <c r="J20" s="17">
+        <v>25.9</v>
+      </c>
+      <c r="K20" s="20">
+        <v>16384</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="20"/>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="36" t="s">
+      <c r="D22" s="36">
+        <v>16</v>
+      </c>
+      <c r="E22" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="36">
-        <v>16</v>
-      </c>
-      <c r="E20" s="36" t="s">
+      <c r="F22" s="37">
+        <v>3.2829999999999999E-3</v>
+      </c>
+      <c r="G22" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="F20" s="37">
-        <v>3.2829999999999999E-3</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="H20" s="39">
+      <c r="H22" s="39">
         <v>6.8992999999999999E-2</v>
       </c>
-      <c r="I20" s="40">
+      <c r="I22" s="40">
         <v>272.11</v>
       </c>
-      <c r="J20" s="41">
+      <c r="J22" s="41">
         <v>487.14</v>
       </c>
-      <c r="K20" s="42">
+      <c r="K22" s="42">
         <v>34222.300000000003</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
-      <c r="B21" s="10"/>
+    <row r="23" spans="1:11">
+      <c r="B23" s="10"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" sqref="C2:C12 C14:C20" xr:uid="{C300DFF5-46E8-4F25-B753-4EE6C8F7C280}">
+    <dataValidation type="list" sqref="C2:C12 C16:C22" xr:uid="{C300DFF5-46E8-4F25-B753-4EE6C8F7C280}">
       <formula1>"100%=1 núcleo,100%=capacidad total"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B2:B21" xr:uid="{1AD00D99-B2BA-4FAF-B153-E405C90E461E}">
+    <dataValidation type="list" sqref="B2:B23" xr:uid="{1AD00D99-B2BA-4FAF-B153-E405C90E461E}">
       <formula1>"psutil,ps + jcmd,ps,Otro"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C13" xr:uid="{4B57103C-9F02-483C-9123-35C9E0AB2911}">
+    <dataValidation type="list" allowBlank="1" sqref="C13:C15" xr:uid="{4B57103C-9F02-483C-9123-35C9E0AB2911}">
       <formula1>"100%=1 núcleo,100%=capacidad total"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1238,7 +1414,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="21.1796875" customWidth="1"/>
@@ -1458,73 +1634,131 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>41</v>
+      <c r="A14" s="55" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="56" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" t="s">
-        <v>42</v>
+      <c r="A15" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="56" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>43</v>
+      <c r="A16" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="56" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="56" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="50" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="50" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="50" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>38</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="43" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="43" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="34" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="43" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="43" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1535,7 +1769,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="23.08984375" customWidth="1"/>
@@ -1718,64 +1952,110 @@
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="A14" s="55" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="55">
+        <v>1</v>
+      </c>
+      <c r="D14" s="55">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="55">
+        <v>1</v>
+      </c>
+      <c r="D15" s="55">
+        <v>812000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="55">
+        <v>1</v>
+      </c>
+      <c r="D16" s="55">
+        <v>249000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="58">
+      <c r="A17" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="24">
-        <v>3</v>
-      </c>
-      <c r="D17" s="24">
-        <v>160787</v>
+      <c r="B17" s="51" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17">
+        <v>12</v>
+      </c>
+      <c r="D17">
+        <v>16466877</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18" s="35">
-        <v>86900</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>38</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="24">
+        <v>3</v>
+      </c>
+      <c r="D19" s="24">
+        <v>160787</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20" s="35">
+        <v>86900</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C20" s="45">
+      <c r="C22" s="45">
         <v>10</v>
       </c>
-      <c r="D20" s="45">
+      <c r="D22" s="45">
         <v>47577</v>
       </c>
     </row>
@@ -1786,7 +2066,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49169CDD-39DA-43A4-BA10-B1D9578FCAE5}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="21.1796875" customWidth="1"/>
@@ -1800,13 +2080,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1909,64 +2189,110 @@
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>41</v>
+      <c r="A14" s="57" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="57" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>42</v>
+      <c r="A15" s="57" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>43</v>
+      <c r="A16" s="57" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="57" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="48" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="48" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>38</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="46" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="46" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="46" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
se agregaron más proyectos del 2° Cuatrimestre del 2026 de PROGC
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_pc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\medidor de metricas\automatizacion_completa\datos_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010CA5AE-4F4B-4F5E-B6A4-7839BC2EFF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A0BB1C-6E6D-44E0-A845-DE2E7E0D2320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CPU_Memoria" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="75">
   <si>
     <t>Codigo</t>
   </si>
@@ -258,6 +258,12 @@
   </si>
   <si>
     <t>114.2%</t>
+  </si>
+  <si>
+    <t>Simulación estándar (4 workers, 50 cuentas, 8M transf.)</t>
+  </si>
+  <si>
+    <t>Estrés alta contención (16 workers, 2 cuentas, 8M transf.)</t>
   </si>
 </sst>
 </file>
@@ -370,14 +376,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -530,11 +537,37 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
     <cellStyle name="Millares" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Millares 2" xfId="3" xr:uid="{C5AA9BD5-CEF8-4E4C-AD7A-A41F277842E7}"/>
     <cellStyle name="Millares 3" xfId="4" xr:uid="{FF52AADE-9C35-4158-BE53-F76058096985}"/>
+    <cellStyle name="Millares 4" xfId="5" xr:uid="{68E4274D-0B58-40F9-A683-07203EE2A7DC}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{0352F441-D3BB-49AE-B4AD-2AF916746F23}"/>
   </cellStyles>
@@ -1261,16 +1294,36 @@
       <c r="A18" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="20"/>
+      <c r="B18" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="61">
+        <v>2</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" s="62">
+        <v>1.272</v>
+      </c>
+      <c r="G18" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="H18" s="63">
+        <v>1.0149999999999999</v>
+      </c>
+      <c r="I18" s="64">
+        <v>103.9</v>
+      </c>
+      <c r="J18" s="65">
+        <v>104.7</v>
+      </c>
+      <c r="K18" s="66">
+        <v>8030</v>
+      </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" t="s">
@@ -1705,6 +1758,18 @@
       <c r="A18" t="s">
         <v>42</v>
       </c>
+      <c r="B18" s="58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="58" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="58" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
@@ -2011,6 +2076,15 @@
       <c r="A18" t="s">
         <v>42</v>
       </c>
+      <c r="B18" s="60" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
+      </c>
+      <c r="D18">
+        <v>13348</v>
+      </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
@@ -2248,6 +2322,15 @@
       <c r="A18" t="s">
         <v>42</v>
       </c>
+      <c r="B18" s="59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="59" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="59" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">

</xml_diff>